<commit_message>
CM and CWM analysis updated with reduced datset of traits Removing additional plot not needed New Supplementary folder in results Script updating and cleaning
</commit_message>
<xml_diff>
--- a/results/mcmc model results.xlsx
+++ b/results/mcmc model results.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="49">
   <si>
     <t>MCMC-GLMM</t>
   </si>
@@ -185,16 +185,13 @@
   </si>
   <si>
     <t>species (ID)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -209,6 +206,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Lucida Sans Typewriter"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Lucida Sans Typewriter"/>
       <family val="3"/>
     </font>
@@ -381,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -403,13 +406,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -449,7 +455,7 @@
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0AFD21C-D7B4-FB1B-220E-B914D6018E3C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{D0AFD21C-D7B4-FB1B-220E-B914D6018E3C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -498,7 +504,7 @@
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86617454-A19B-5877-3938-2280222424CC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{86617454-A19B-5877-3938-2280222424CC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -542,7 +548,7 @@
         <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA12731C-8F12-9DF7-E6C7-8950A41B37BA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{AA12731C-8F12-9DF7-E6C7-8950A41B37BA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -908,10 +914,10 @@
       <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="15"/>
+      <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:12" ht="15" thickBot="1">
       <c r="A2" s="1"/>
@@ -937,23 +943,23 @@
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="1">
-        <v>-1.9919800000000001</v>
+        <v>-2.0389900000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>-3.54175</v>
+        <v>-3.63686</v>
       </c>
       <c r="E3" s="1">
-        <v>-0.41058</v>
+        <v>-0.57831999999999995</v>
       </c>
       <c r="F3" s="1">
-        <v>8863</v>
+        <v>8418</v>
       </c>
       <c r="G3" s="1">
-        <v>1.1299999999999999E-2</v>
+        <v>1.0888999999999999E-2</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>7</v>
@@ -975,61 +981,61 @@
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="1">
-        <v>-0.82526999999999995</v>
+        <v>-1.5566199999999999</v>
       </c>
       <c r="D4" s="1">
-        <v>-1.66628</v>
+        <v>-2.4574500000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>4.546E-2</v>
+        <v>-0.63407000000000002</v>
       </c>
       <c r="F4" s="1">
-        <v>9593</v>
+        <v>9234</v>
       </c>
       <c r="G4" s="1">
-        <v>5.7599999999999998E-2</v>
+        <v>8.8900000000000003E-4</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>46</v>
       </c>
       <c r="J4" s="10">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="K4" s="10">
         <v>0</v>
       </c>
       <c r="L4" s="11">
-        <v>0.82</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1">
-        <v>-2.1088900000000002</v>
+        <v>-2.1186600000000002</v>
       </c>
       <c r="D5" s="1">
-        <v>-3.0248900000000001</v>
+        <v>-3.0167899999999999</v>
       </c>
       <c r="E5" s="1">
-        <v>-1.2336800000000001</v>
+        <v>-1.1714599999999999</v>
       </c>
       <c r="F5" s="1">
-        <v>8676</v>
+        <v>8683</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>11</v>
@@ -1038,70 +1044,70 @@
         <v>47</v>
       </c>
       <c r="J5" s="10">
-        <v>1.73</v>
+        <v>1.39</v>
       </c>
       <c r="K5" s="10">
         <v>0</v>
       </c>
       <c r="L5" s="11">
-        <v>7.11</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="1">
-        <v>0.42010999999999998</v>
+        <v>0.42198000000000002</v>
       </c>
       <c r="D6" s="1">
-        <v>-0.36038999999999999</v>
+        <v>-0.44395000000000001</v>
       </c>
       <c r="E6" s="1">
-        <v>1.2763500000000001</v>
+        <v>1.2272799999999999</v>
       </c>
       <c r="F6" s="1">
         <v>9000</v>
       </c>
       <c r="G6" s="1">
-        <v>0.30669999999999997</v>
+        <v>0.32911099999999999</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="9" t="s">
         <v>48</v>
       </c>
       <c r="J6" s="10">
-        <v>8.2200000000000006</v>
+        <v>9.0299999999999994</v>
       </c>
       <c r="K6" s="10">
-        <v>3.79</v>
+        <v>4.5199999999999996</v>
       </c>
       <c r="L6" s="11">
-        <v>13.22</v>
+        <v>14.33</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" thickBot="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="1">
-        <v>0.41213</v>
+        <v>0.41521000000000002</v>
       </c>
       <c r="D7" s="1">
-        <v>-0.80940999999999996</v>
+        <v>-0.83374000000000004</v>
       </c>
       <c r="E7" s="1">
-        <v>1.7115100000000001</v>
+        <v>1.73888</v>
       </c>
       <c r="F7" s="1">
         <v>9000</v>
       </c>
       <c r="G7" s="1">
-        <v>0.51359999999999995</v>
+        <v>0.52444400000000002</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="12"/>
@@ -1111,45 +1117,45 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="1"/>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="1">
-        <v>0.50585000000000002</v>
+        <v>0.57179000000000002</v>
       </c>
       <c r="D8" s="1">
-        <v>-0.70916000000000001</v>
+        <v>-0.61851</v>
       </c>
       <c r="E8" s="1">
-        <v>1.6048</v>
+        <v>1.8295300000000001</v>
       </c>
       <c r="F8" s="1">
-        <v>9000</v>
+        <v>9067</v>
       </c>
       <c r="G8" s="1">
-        <v>0.39019999999999999</v>
+        <v>0.34799999999999998</v>
       </c>
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="1"/>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="18" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="1">
-        <v>-1.1674899999999999</v>
+        <v>-1.22404</v>
       </c>
       <c r="D9" s="1">
-        <v>-2.36049</v>
+        <v>-2.4805899999999999</v>
       </c>
       <c r="E9" s="1">
-        <v>0.11910999999999999</v>
+        <v>2.6669999999999999E-2</v>
       </c>
       <c r="F9" s="1">
-        <v>8713</v>
+        <v>9000</v>
       </c>
       <c r="G9" s="1">
-        <v>6.6000000000000003E-2</v>
+        <v>5.7333000000000002E-2</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>29</v>
@@ -1157,23 +1163,23 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="1"/>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="18" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="1">
-        <v>-0.17247999999999999</v>
+        <v>-0.18956000000000001</v>
       </c>
       <c r="D10" s="1">
-        <v>-1.2813699999999999</v>
+        <v>-1.30114</v>
       </c>
       <c r="E10" s="1">
-        <v>0.93318000000000001</v>
+        <v>0.96231999999999995</v>
       </c>
       <c r="F10" s="1">
         <v>9000</v>
       </c>
       <c r="G10" s="1">
-        <v>0.75509999999999999</v>
+        <v>0.74622200000000005</v>
       </c>
       <c r="H10" s="1"/>
     </row>
@@ -1208,10 +1214,10 @@
       <c r="B2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="15"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="1"/>
@@ -1249,30 +1255,30 @@
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="1">
-        <v>-1.2244999999999999</v>
+        <v>-1.3229</v>
       </c>
       <c r="D4" s="1">
-        <v>-3.1375999999999999</v>
+        <v>-3.2982</v>
       </c>
       <c r="E4" s="1">
-        <v>0.65390000000000004</v>
+        <v>0.56210000000000004</v>
       </c>
       <c r="F4" s="1">
-        <v>10585</v>
+        <v>9000</v>
       </c>
       <c r="G4" s="1">
-        <v>0.17499999999999999</v>
+        <v>0.1464</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="9" t="s">
         <v>46</v>
       </c>
       <c r="J4" s="10">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="K4" s="10">
         <v>0</v>
@@ -1285,56 +1291,58 @@
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="1">
-        <v>-0.33179999999999998</v>
+        <v>-0.99890000000000001</v>
       </c>
       <c r="D5" s="1">
-        <v>-1.1899</v>
+        <v>-1.8089999999999999</v>
       </c>
       <c r="E5" s="1">
-        <v>0.4622</v>
+        <v>-0.10340000000000001</v>
       </c>
       <c r="F5" s="1">
         <v>9000</v>
       </c>
       <c r="G5" s="1">
-        <v>0.437</v>
-      </c>
-      <c r="H5" s="1"/>
+        <v>2.1299999999999999E-2</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="I5" s="9" t="s">
         <v>47</v>
       </c>
       <c r="J5" s="10">
-        <v>3.86</v>
+        <v>3.85</v>
       </c>
       <c r="K5" s="10">
         <v>0</v>
       </c>
       <c r="L5" s="11">
-        <v>14.38</v>
+        <v>14.71</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="1">
-        <v>-3.3443999999999998</v>
+        <v>-3.4032</v>
       </c>
       <c r="D6" s="1">
-        <v>-4.2708000000000004</v>
+        <v>-4.3212999999999999</v>
       </c>
       <c r="E6" s="1">
-        <v>-2.3973</v>
+        <v>-2.4544999999999999</v>
       </c>
       <c r="F6" s="1">
-        <v>9000</v>
+        <v>8832</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>10</v>
@@ -1346,36 +1354,36 @@
         <v>48</v>
       </c>
       <c r="J6" s="10">
-        <v>6.89</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>49</v>
+        <v>7.76</v>
+      </c>
+      <c r="K6" s="10">
+        <v>0</v>
       </c>
       <c r="L6" s="11">
-        <v>13.01</v>
+        <v>14.42</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" thickBot="1">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="1">
-        <v>0.24379999999999999</v>
+        <v>0.2477</v>
       </c>
       <c r="D7" s="1">
-        <v>-0.59450000000000003</v>
+        <v>-0.56359999999999999</v>
       </c>
       <c r="E7" s="1">
-        <v>1.0278</v>
+        <v>1.0818000000000001</v>
       </c>
       <c r="F7" s="1">
         <v>9000</v>
       </c>
       <c r="G7" s="1">
-        <v>0.55600000000000005</v>
+        <v>0.55800000000000005</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="12"/>
@@ -1395,10 +1403,10 @@
       <c r="B12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="15"/>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="1"/>
@@ -1436,23 +1444,23 @@
       <c r="A14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="17">
-        <v>-2.2745299999999999</v>
+      <c r="C14" s="15">
+        <v>-2.2702</v>
       </c>
       <c r="D14" s="1">
-        <v>-5.1882099999999998</v>
+        <v>-5.1426999999999996</v>
       </c>
       <c r="E14" s="1">
-        <v>0.39273000000000002</v>
+        <v>0.34660000000000002</v>
       </c>
       <c r="F14" s="1">
-        <v>8605</v>
+        <v>9000</v>
       </c>
       <c r="G14" s="1">
-        <v>7.8200000000000006E-2</v>
+        <v>7.7556E-2</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>29</v>
@@ -1461,74 +1469,74 @@
         <v>46</v>
       </c>
       <c r="J14" s="10">
-        <v>6.9000000000000006E-2</v>
+        <v>0.69</v>
       </c>
       <c r="K14" s="10">
         <v>0.04</v>
       </c>
       <c r="L14" s="11">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="17">
-        <v>-0.71604000000000001</v>
+      <c r="C15" s="15">
+        <v>-1.4044000000000001</v>
       </c>
       <c r="D15" s="1">
-        <v>-1.4507000000000001</v>
+        <v>-2.1480000000000001</v>
       </c>
       <c r="E15" s="1">
-        <v>-6.2710000000000002E-2</v>
+        <v>-0.69299999999999995</v>
       </c>
       <c r="F15" s="1">
-        <v>8680</v>
+        <v>9440</v>
       </c>
       <c r="G15" s="1">
-        <v>4.1300000000000003E-2</v>
+        <v>2.22E-4</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>47</v>
       </c>
       <c r="J15" s="10">
-        <v>7.76</v>
+        <v>7.85</v>
       </c>
       <c r="K15" s="10">
         <v>0</v>
       </c>
       <c r="L15" s="11">
-        <v>26.25</v>
+        <v>26.77</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="17">
-        <v>-2.0085799999999998</v>
+      <c r="C16" s="15">
+        <v>-2.0310999999999999</v>
       </c>
       <c r="D16" s="1">
-        <v>-2.7261799999999998</v>
+        <v>-2.8205</v>
       </c>
       <c r="E16" s="1">
-        <v>-1.2743</v>
+        <v>-1.2966</v>
       </c>
       <c r="F16" s="1">
         <v>9000</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>11</v>
@@ -1537,36 +1545,36 @@
         <v>48</v>
       </c>
       <c r="J16" s="10">
-        <v>7.29</v>
+        <v>7.47</v>
       </c>
       <c r="K16" s="10">
         <v>0</v>
       </c>
       <c r="L16" s="11">
-        <v>16.97</v>
+        <v>17.309999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15" thickBot="1">
       <c r="A17" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="17">
-        <v>0.47788000000000003</v>
+      <c r="C17" s="15">
+        <v>0.4592</v>
       </c>
       <c r="D17" s="1">
-        <v>-0.17923</v>
+        <v>-0.21690000000000001</v>
       </c>
       <c r="E17" s="1">
-        <v>1.12344</v>
+        <v>1.1177999999999999</v>
       </c>
       <c r="F17" s="1">
         <v>9000</v>
       </c>
       <c r="G17" s="1">
-        <v>0.1462</v>
+        <v>0.17955599999999999</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="12"/>
@@ -1603,10 +1611,10 @@
       <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16"/>
+      <c r="D1" s="17"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -1851,10 +1859,10 @@
       <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16"/>
+      <c r="D1" s="17"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>

</xml_diff>